<commit_message>
feat: add support for short answer questions in schema, forms, and UI components
</commit_message>
<xml_diff>
--- a/public/templates/template-impor-soal.xlsx
+++ b/public/templates/template-impor-soal.xlsx
@@ -397,7 +397,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:P4"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="23.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,12 +455,15 @@
         <v>kunci</v>
       </c>
       <c r="M1" t="str">
+        <v>kunci_jawaban_singkat</v>
+      </c>
+      <c r="N1" t="str">
         <v>pedoman</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>rubrik</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>ada_gambar</v>
       </c>
     </row>
@@ -465,16 +486,16 @@
       <c r="F2">
         <v>-1</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="str">
         <v>3</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="str">
         <v>4</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="str">
         <v>5</v>
       </c>
-      <c r="J2">
+      <c r="J2" t="str">
         <v>6</v>
       </c>
       <c r="K2" t="str">
@@ -489,7 +510,10 @@
       <c r="N2" t="str">
         <v/>
       </c>
-      <c r="O2">
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2">
         <v>0</v>
       </c>
     </row>
@@ -531,18 +555,71 @@
         <v/>
       </c>
       <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
         <v>Fotosintesis adalah proses tumbuhan mengubah cahaya, air, dan CO2 menjadi glukosa.</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>Skor penuh jika menyebut cahaya, air, CO2, dan hasil glukosa.</v>
       </c>
-      <c r="O3">
+      <c r="P3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Paket Matematika</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Contoh</v>
+      </c>
+      <c r="C4" t="str">
+        <v>jawaban singkat</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Ibu kota Indonesia adalah...</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>-1</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>jakarta</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>